<commit_message>
Update Integrated Disclosure 2026-03-04
</commit_message>
<xml_diff>
--- a/Integrated_Disclosure_Report.xlsx
+++ b/Integrated_Disclosure_Report.xlsx
@@ -570,7 +570,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
+          <t xml:space="preserve">[기재정정]단일판매ㆍ공급계약체결              </t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -584,19 +584,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>10676552100</v>
+        <v>10104945135</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>10676552100</v>
+        <v>10104945135</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>17.92</v>
+        <v>16.96</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">

</xml_diff>

<commit_message>
Update Integrated Disclosure 2026-07-01
</commit_message>
<xml_diff>
--- a/Integrated_Disclosure_Report.xlsx
+++ b/Integrated_Disclosure_Report.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -570,12 +570,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">[기재정정]단일판매ㆍ공급계약체결              </t>
+          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
+          <t>데이터센터용슈퍼커패시터시스템공급계약</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -584,45 +584,45 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>10104945135</v>
+        <v>41215393800</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>10104945135</v>
+        <v>41215393800</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>16.96</v>
+        <v>50.12</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ACBELPOLYTECHINC</t>
+          <t>BloomEnergyCorporation</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2027-04-10</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
+          <t xml:space="preserve">[기재정정]단일판매ㆍ공급계약체결              </t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -636,36 +636,88 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6758155342</v>
+        <v>10104945135</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>6758155342</v>
+        <v>10104945135</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ACBELPOLYTECHINC</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>미해당</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>6758155342</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>6758155342</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
         <v>11.34</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>ACBELPOLYTECHINC</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>2025-06-13</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2025-09-30</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2025-06-13</t>
         </is>

</xml_diff>

<commit_message>
Update Integrated Disclosure 2026-07-07
</commit_message>
<xml_diff>
--- a/Integrated_Disclosure_Report.xlsx
+++ b/Integrated_Disclosure_Report.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -575,7 +575,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>데이터센터용슈퍼커패시터시스템공급계약</t>
+          <t>데이터센터용슈퍼커패시터공급계약</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -584,50 +584,50 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>41215393800</v>
+        <v>13112996702</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>41215393800</v>
+        <v>13112996702</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>50.12</v>
+        <v>15.95</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>BloomEnergyCorporation</t>
+          <t>SANMINACORPORATION</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2027-04-10</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">[기재정정]단일판매ㆍ공급계약체결              </t>
+          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
+          <t>데이터센터용슈퍼커패시터시스템공급계약</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -636,45 +636,45 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>10104945135</v>
+        <v>41215393800</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>10104945135</v>
+        <v>41215393800</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>16.96</v>
+        <v>50.12</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ACBELPOLYTECHINC</t>
+          <t>BloomEnergyCorporation</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2027-04-10</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
+          <t xml:space="preserve">[기재정정]단일판매ㆍ공급계약체결              </t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -688,36 +688,88 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6758155342</v>
+        <v>10104945135</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>6758155342</v>
+        <v>10104945135</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ACBELPOLYTECHINC</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>미해당</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6758155342</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>6758155342</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
         <v>11.34</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>ACBELPOLYTECHINC</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>2025-06-13</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2025-09-30</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2025-06-13</t>
         </is>

</xml_diff>

<commit_message>
Update Integrated Disclosure 2026-07-13
</commit_message>
<xml_diff>
--- a/Integrated_Disclosure_Report.xlsx
+++ b/Integrated_Disclosure_Report.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>13112996702</v>
+        <v>38361874110</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>13112996702</v>
+        <v>38361874110</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>15.95</v>
+        <v>46.65</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>SANMINACORPORATION</t>
+          <t>ACBELPOLYTECHINC</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2027-03-15</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>데이터센터용슈퍼커패시터시스템공급계약</t>
+          <t>데이터센터용슈퍼커패시터공급계약</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -636,50 +636,50 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>41215393800</v>
+        <v>13112996702</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>41215393800</v>
+        <v>13112996702</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>50.12</v>
+        <v>15.95</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>BloomEnergyCorporation</t>
+          <t>SANMINACORPORATION</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2027-04-10</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">[기재정정]단일판매ㆍ공급계약체결              </t>
+          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
+          <t>데이터센터용슈퍼커패시터시스템공급계약</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -688,88 +688,140 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>10104945135</v>
+        <v>41215393800</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>10104945135</v>
+        <v>41215393800</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>16.96</v>
+        <v>50.12</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ACBELPOLYTECHINC</t>
+          <t>BloomEnergyCorporation</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2027-04-10</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t xml:space="preserve">[기재정정]단일판매ㆍ공급계약체결              </t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>미해당</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>10104945135</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>10104945135</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>ACBELPOLYTECHINC</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>미해당</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D6" t="n">
         <v>6758155342</v>
       </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="n">
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
         <v>6758155342</v>
       </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
         <v>11.34</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>ACBELPOLYTECHINC</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>2025-06-13</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>2025-09-30</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>2025-06-13</t>
         </is>

</xml_diff>

<commit_message>
Update Integrated Disclosure 2026-09-08
</commit_message>
<xml_diff>
--- a/Integrated_Disclosure_Report.xlsx
+++ b/Integrated_Disclosure_Report.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>38361874110</v>
+        <v>13300418504</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>38361874110</v>
+        <v>13300418504</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>46.65</v>
+        <v>16.17</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ACBELPOLYTECHINC</t>
+          <t>SANMINACORPORATION</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2027-03-15</t>
+          <t>2027-01-28</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
@@ -636,38 +636,38 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>13112996702</v>
+        <v>38361874110</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>13112996702</v>
+        <v>38361874110</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>15.95</v>
+        <v>46.65</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>SANMINACORPORATION</t>
+          <t>ACBELPOLYTECHINC</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2027-03-15</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>데이터센터용슈퍼커패시터시스템공급계약</t>
+          <t>데이터센터용슈퍼커패시터공급계약</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -688,50 +688,50 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>41215393800</v>
+        <v>13112996702</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>41215393800</v>
+        <v>13112996702</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>50.12</v>
+        <v>15.95</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>BloomEnergyCorporation</t>
+          <t>SANMINACORPORATION</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2027-04-10</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">[기재정정]단일판매ㆍ공급계약체결              </t>
+          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
+          <t>데이터센터용슈퍼커패시터시스템공급계약</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -740,88 +740,140 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>10104945135</v>
+        <v>41215393800</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>10104945135</v>
+        <v>41215393800</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>16.96</v>
+        <v>50.12</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>ACBELPOLYTECHINC</t>
+          <t>BloomEnergyCorporation</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2027-04-10</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t xml:space="preserve">[기재정정]단일판매ㆍ공급계약체결              </t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>미해당</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>10104945135</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>10104945135</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>ACBELPOLYTECHINC</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>미해당</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D7" t="n">
         <v>6758155342</v>
       </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
         <v>6758155342</v>
       </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
         <v>11.34</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>ACBELPOLYTECHINC</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>2025-06-13</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>2025-09-30</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>2025-06-13</t>
         </is>

</xml_diff>